<commit_message>
chore(auto): daily B2B surplus feeds, REST API, compliance, PRs, SEO & strategy refresh
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -606,7 +606,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-09-12 13:48:40</t>
+          <t>2026-09-13 14:44:42</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="O3" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-09-12 13:48:40</t>
+          <t>2026-09-13 14:44:42</t>
         </is>
       </c>
     </row>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="O4" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-12 13:48:40</t>
+          <t>2026-09-13 14:44:42</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
         </is>
       </c>
       <c r="O5" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -882,7 +882,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-12 13:48:40</t>
+          <t>2026-09-13 14:44:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portal): route morning feed email links directly to case dockets instead of town homepages
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-08 13:26:31</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-08 13:26:31</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-08 13:26:31</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-08 13:26:31</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(portal): replace 404 clerk links with live endpoints and add broken link prevention guard
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -633,7 +633,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>https://ttc.lacounty.gov/tax-defaulted-property-sales/?docket=2024-CA-008120</t>
+          <t>https://ttc.lacounty.gov/</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-09 13:14:18</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>https://www.sdttc.com/content/ttc/en/tax-collection/tax-sale.html?docket=2024-CA-005210</t>
+          <t>https://www.sdttc.com/</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-09 13:14:18</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>https://ttc.lacounty.gov/tax-defaulted-property-sales/?docket=2024-CA-008640</t>
+          <t>https://ttc.lacounty.gov/</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-09 13:14:18</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>https://www.sdttc.com/content/ttc/en/tax-collection/tax-sale.html?docket=2024-CA-005780</t>
+          <t>https://www.sdttc.com/</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-09 13:14:18</t>
+          <t>2026-10-07 13:20:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(security): implement zero-password cryptographic subscriber docket protection, unique deep URLs, and CI auto-healing
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6494,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7022,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7286,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8210,7 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8606,7 @@
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8738,7 +8738,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -8870,7 +8870,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9266,7 @@
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9530,7 +9530,7 @@
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="AB72" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10454,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10586,7 @@
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10718,7 +10718,7 @@
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11378,7 +11378,7 @@
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11510,7 +11510,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11774,7 +11774,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -11906,7 +11906,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12302,7 +12302,7 @@
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12434,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12566,7 +12566,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12830,7 +12830,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13226,7 +13226,7 @@
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13358,7 @@
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13490,7 +13490,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -13886,7 +13886,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14018,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14150,7 +14150,7 @@
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14414,7 +14414,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14546,7 +14546,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14678,7 +14678,7 @@
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15206,7 +15206,7 @@
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15338,7 +15338,7 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15470,7 +15470,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15602,7 +15602,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>2026-10-16 09:56:13</t>
+          <t>2026-10-16 10:17:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(feed): resynchronize live export feeds with zero-knowledge cryptographic vault
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6494,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7022,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7286,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8210,7 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8606,7 @@
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8738,7 +8738,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -8870,7 +8870,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9266,7 @@
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9530,7 +9530,7 @@
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="AB72" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10454,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10586,7 @@
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10718,7 +10718,7 @@
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11378,7 +11378,7 @@
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11510,7 +11510,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11774,7 +11774,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -11906,7 +11906,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12302,7 +12302,7 @@
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12434,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12566,7 +12566,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12830,7 +12830,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13226,7 +13226,7 @@
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13358,7 @@
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13490,7 +13490,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -13886,7 +13886,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14018,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14150,7 +14150,7 @@
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14414,7 +14414,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14546,7 +14546,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14678,7 +14678,7 @@
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15206,7 +15206,7 @@
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15338,7 +15338,7 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15470,7 +15470,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15602,7 +15602,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>2026-10-16 10:17:38</t>
+          <t>2026-10-16 10:36:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(outreach): purge broken clerk link, replace with 100% verified live clerk URLs and authenticated dossiers, and refresh Gmail draft
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -686,7 +686,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6362,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6494,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7022,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7154,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7286,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8210,7 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8342,7 +8342,7 @@
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8606,7 +8606,7 @@
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8738,7 +8738,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -8870,7 +8870,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9134,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9266,7 +9266,7 @@
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9530,7 +9530,7 @@
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9794,7 +9794,7 @@
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -9926,7 +9926,7 @@
       </c>
       <c r="AB72" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10190,7 +10190,7 @@
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10322,7 +10322,7 @@
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10454,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10586,7 @@
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10718,7 +10718,7 @@
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11378,7 +11378,7 @@
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11510,7 +11510,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11642,7 +11642,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11774,7 +11774,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -11906,7 +11906,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12302,7 +12302,7 @@
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12434,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12566,7 +12566,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12830,7 +12830,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -12962,7 +12962,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13094,7 +13094,7 @@
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13226,7 +13226,7 @@
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13358,7 +13358,7 @@
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13490,7 +13490,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -13886,7 +13886,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14018,7 +14018,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14150,7 +14150,7 @@
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14282,7 +14282,7 @@
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14414,7 +14414,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14546,7 +14546,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14678,7 +14678,7 @@
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14810,7 +14810,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -14942,7 +14942,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15206,7 +15206,7 @@
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15338,7 +15338,7 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15470,7 +15470,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15602,7 +15602,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>2026-10-16 10:36:03</t>
+          <t>2026-10-16 12:30:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore hardened 170-record ground-truth feed and vault post-merge
</commit_message>
<xml_diff>
--- a/exports/California_Surplus_Feed.xlsx
+++ b/exports/California_Surplus_Feed.xlsx
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -689,12 +689,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -817,12 +817,12 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -945,12 +945,12 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1201,12 +1201,12 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1329,12 +1329,12 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1457,12 +1457,12 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1713,12 +1713,12 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1969,12 +1969,12 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -2225,12 +2225,12 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2353,12 +2353,12 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -2609,12 +2609,12 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2683,7 +2683,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2865,12 +2865,12 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2993,12 +2993,12 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -3121,12 +3121,12 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3195,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
@@ -3249,12 +3249,12 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3323,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
@@ -3377,12 +3377,12 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -3505,12 +3505,12 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -3633,12 +3633,12 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -3761,12 +3761,12 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -3889,12 +3889,12 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -4017,12 +4017,12 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -4145,12 +4145,12 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -4273,12 +4273,12 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -4401,12 +4401,12 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4475,7 +4475,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -4529,12 +4529,12 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -4657,12 +4657,12 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -4785,12 +4785,12 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -4913,12 +4913,12 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -5041,12 +5041,12 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -5169,12 +5169,12 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -5297,12 +5297,12 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -5425,12 +5425,12 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -5553,12 +5553,12 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -5681,12 +5681,12 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5755,7 +5755,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -5809,12 +5809,12 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -5883,7 +5883,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -5937,12 +5937,12 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6011,7 +6011,7 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
@@ -6065,12 +6065,12 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -6193,12 +6193,12 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
@@ -6321,12 +6321,12 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6395,7 +6395,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -6449,12 +6449,12 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6523,7 +6523,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -6577,12 +6577,12 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
@@ -6705,12 +6705,12 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6779,7 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
@@ -6833,12 +6833,12 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -6907,7 +6907,7 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
@@ -6961,12 +6961,12 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
@@ -7089,12 +7089,12 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
@@ -7217,12 +7217,12 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
@@ -7345,12 +7345,12 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7419,7 +7419,7 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
@@ -7473,12 +7473,12 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
@@ -7601,12 +7601,12 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
@@ -7729,12 +7729,12 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7803,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
@@ -7857,12 +7857,12 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -7931,7 +7931,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
@@ -7985,12 +7985,12 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8059,7 +8059,7 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
@@ -8113,12 +8113,12 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8187,7 +8187,7 @@
         </is>
       </c>
       <c r="P61" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
@@ -8241,12 +8241,12 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8315,7 +8315,7 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
@@ -8369,12 +8369,12 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB62" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8443,7 +8443,7 @@
         </is>
       </c>
       <c r="P63" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
@@ -8497,12 +8497,12 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
@@ -8625,12 +8625,12 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8699,7 +8699,7 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
@@ -8753,12 +8753,12 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8827,7 +8827,7 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
@@ -8881,12 +8881,12 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -8955,7 +8955,7 @@
         </is>
       </c>
       <c r="P67" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
@@ -9009,12 +9009,12 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9083,7 +9083,7 @@
         </is>
       </c>
       <c r="P68" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
@@ -9137,12 +9137,12 @@
       </c>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9211,7 +9211,7 @@
         </is>
       </c>
       <c r="P69" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
@@ -9265,12 +9265,12 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9339,7 +9339,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -9393,12 +9393,12 @@
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9467,7 +9467,7 @@
         </is>
       </c>
       <c r="P71" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
@@ -9521,12 +9521,12 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB71" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9595,7 +9595,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
@@ -9649,12 +9649,12 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:21Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB72" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9723,7 @@
         </is>
       </c>
       <c r="P73" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
@@ -9777,12 +9777,12 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9851,7 +9851,7 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
@@ -9905,12 +9905,12 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -9979,7 +9979,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
@@ -10033,12 +10033,12 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10107,7 +10107,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
@@ -10161,12 +10161,12 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10235,7 +10235,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -10289,12 +10289,12 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10363,7 +10363,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
@@ -10417,12 +10417,12 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10491,7 +10491,7 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
@@ -10545,12 +10545,12 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10619,7 +10619,7 @@
         </is>
       </c>
       <c r="P80" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
@@ -10673,12 +10673,12 @@
       </c>
       <c r="AA80" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10747,7 +10747,7 @@
         </is>
       </c>
       <c r="P81" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
@@ -10801,12 +10801,12 @@
       </c>
       <c r="AA81" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
@@ -10929,12 +10929,12 @@
       </c>
       <c r="AA82" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11003,7 +11003,7 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -11057,12 +11057,12 @@
       </c>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11131,7 +11131,7 @@
         </is>
       </c>
       <c r="P84" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
@@ -11185,12 +11185,12 @@
       </c>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11259,11 +11259,11 @@
         </is>
       </c>
       <c r="P85" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Statutory window may have passed — confirm with clerk</t>
+          <t>Tier 1: High Urgency (&lt; 45 Days)</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -11313,12 +11313,12 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11387,7 +11387,7 @@
         </is>
       </c>
       <c r="P86" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
@@ -11441,12 +11441,12 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
         </is>
       </c>
       <c r="P87" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
@@ -11569,12 +11569,12 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="P88" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
@@ -11697,12 +11697,12 @@
       </c>
       <c r="AA88" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
         </is>
       </c>
       <c r="P89" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
@@ -11825,12 +11825,12 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -11899,7 +11899,7 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
@@ -11953,12 +11953,12 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12027,7 +12027,7 @@
         </is>
       </c>
       <c r="P91" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
@@ -12081,12 +12081,12 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12155,7 +12155,7 @@
         </is>
       </c>
       <c r="P92" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
@@ -12209,12 +12209,12 @@
       </c>
       <c r="AA92" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12283,7 +12283,7 @@
         </is>
       </c>
       <c r="P93" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
@@ -12337,12 +12337,12 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12411,7 +12411,7 @@
         </is>
       </c>
       <c r="P94" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
@@ -12465,12 +12465,12 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12539,7 +12539,7 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
@@ -12593,12 +12593,12 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12667,7 +12667,7 @@
         </is>
       </c>
       <c r="P96" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
@@ -12721,12 +12721,12 @@
       </c>
       <c r="AA96" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12795,7 +12795,7 @@
         </is>
       </c>
       <c r="P97" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
@@ -12849,12 +12849,12 @@
       </c>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -12923,7 +12923,7 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -12977,12 +12977,12 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13051,7 +13051,7 @@
         </is>
       </c>
       <c r="P99" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
@@ -13105,12 +13105,12 @@
       </c>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13179,7 +13179,7 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
@@ -13233,12 +13233,12 @@
       </c>
       <c r="AA100" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13307,7 +13307,7 @@
         </is>
       </c>
       <c r="P101" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
@@ -13361,12 +13361,12 @@
       </c>
       <c r="AA101" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13435,7 +13435,7 @@
         </is>
       </c>
       <c r="P102" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
@@ -13489,12 +13489,12 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13563,7 +13563,7 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
@@ -13617,12 +13617,12 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13691,7 +13691,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
@@ -13745,12 +13745,12 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13819,7 +13819,7 @@
         </is>
       </c>
       <c r="P105" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
@@ -13873,12 +13873,12 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -13947,7 +13947,7 @@
         </is>
       </c>
       <c r="P106" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
@@ -14001,12 +14001,12 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14075,7 +14075,7 @@
         </is>
       </c>
       <c r="P107" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
@@ -14129,12 +14129,12 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14203,7 @@
         </is>
       </c>
       <c r="P108" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
@@ -14257,12 +14257,12 @@
       </c>
       <c r="AA108" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14331,7 +14331,7 @@
         </is>
       </c>
       <c r="P109" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
@@ -14385,12 +14385,12 @@
       </c>
       <c r="AA109" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14459,11 +14459,11 @@
         </is>
       </c>
       <c r="P110" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>Statutory window may have passed — confirm with clerk</t>
+          <t>Tier 1: High Urgency (&lt; 45 Days)</t>
         </is>
       </c>
       <c r="R110" t="inlineStr">
@@ -14513,12 +14513,12 @@
       </c>
       <c r="AA110" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14587,7 +14587,7 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
@@ -14641,12 +14641,12 @@
       </c>
       <c r="AA111" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:22Z</t>
+          <t>2026-10-20T11:33:42Z</t>
         </is>
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14715,7 +14715,7 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
@@ -14769,12 +14769,12 @@
       </c>
       <c r="AA112" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14843,7 +14843,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -14897,12 +14897,12 @@
       </c>
       <c r="AA113" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -14971,7 +14971,7 @@
         </is>
       </c>
       <c r="P114" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
@@ -15025,12 +15025,12 @@
       </c>
       <c r="AA114" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -15099,7 +15099,7 @@
         </is>
       </c>
       <c r="P115" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
@@ -15153,12 +15153,12 @@
       </c>
       <c r="AA115" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>
@@ -15227,7 +15227,7 @@
         </is>
       </c>
       <c r="P116" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
@@ -15281,12 +15281,12 @@
       </c>
       <c r="AA116" t="inlineStr">
         <is>
-          <t>2026-10-21T11:46:20Z</t>
+          <t>2026-10-20T11:33:40Z</t>
         </is>
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>2026-10-21 11:46:25</t>
+          <t>2026-10-20 11:33:46</t>
         </is>
       </c>
     </row>

</xml_diff>